<commit_message>
change the spacing for rows and colums
</commit_message>
<xml_diff>
--- a/Evaluation_Question/Evaluation_Questions.xlsx
+++ b/Evaluation_Question/Evaluation_Questions.xlsx
@@ -1,31 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/fb30f5ea8e07144a/Desktop/FYP/Evaluation_Question/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EC2CD244-6A7F-4C96-9B8A-A07873D420BC}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28770" windowHeight="11940" xr2:uid="{3E398CB9-F5B5-44F0-A993-76D53D7D2A13}"/>
+    <workbookView/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet r:id="rId1" name="Sheet1" sheetId="1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="0" iterateCount="100" iterateDelta="0.001"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="105">
   <si>
     <t>ID</t>
   </si>
@@ -345,35 +333,29 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <fonts count="3">
     <font>
+      <b val="0"/>
+      <i val="0"/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="新細明體"/>
-      <family val="2"/>
-      <charset val="136"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <i val="0"/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Segoe UI"/>
-      <family val="2"/>
     </font>
     <font>
-      <b/>
+      <b val="0"/>
+      <i val="0"/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Segoe UI"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <name val="新細明體"/>
-      <family val="2"/>
-      <charset val="136"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -386,7 +368,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF5F5F5"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -414,36 +395,53 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
+      <alignment horizontal="general" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
+      <alignment horizontal="general" vertical="center"/>
     </xf>
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="1"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/featurePropertyBag/featurePropertyBag.xml><?xml version="1.0" encoding="utf-8"?>
+<FeaturePropertyBags xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag">
+  <bag type="Checkbox"/>
+  <bag type="XFControls">
+    <bagId k="CellControl">0</bagId>
+  </bag>
+  <bag type="XFComplement">
+    <bagId k="XFControls">1</bagId>
+  </bag>
+  <bag type="XFComplements" extRef="XFComplementsMapperExtRef">
+    <a k="MappedFeaturePropertyBags">
+      <bagId>2</bagId>
+    </a>
+  </bag>
+  <bag type="DXFComplements" extRef="DXFComplementsMapperExtRef">
+    <a k="MappedFeaturePropertyBags">
+      <bagId>2</bagId>
+    </a>
+  </bag>
+</FeaturePropertyBags>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -489,7 +487,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Calibri Light"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -541,7 +539,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -602,158 +600,183 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="35000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="80000">
               <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
+                <a:alpha val="35000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
-          </a:schemeClr>
-        </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="40000">
               <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
   <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59B07250-27F7-4B6F-9B43-7428E7574E29}">
-  <dimension ref="A1:E76"/>
-  <sheetFormatPr defaultRowHeight="15.75"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{FC0B3B03-EB07-4F2D-B0E4-753680CEB3B8}" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1:G76"/>
+  <sheetFormatPr defaultRowHeight="15.75" defaultColWidth="9.140625" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="1" max="1" width="14.00390625" customWidth="1"/>
     <col min="2" max="2" width="35.7109375" customWidth="1"/>
     <col min="3" max="3" width="21.7109375" customWidth="1"/>
-    <col min="4" max="4" width="21.5703125" customWidth="1"/>
+    <col min="4" max="4" width="21.57421875" customWidth="1"/>
     <col min="5" max="5" width="21.140625" customWidth="1"/>
+    <col min="6" max="7" width="9.140625" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="66.75" thickBot="1">
+    <row r="1" ht="66.75" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -770,7 +793,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="99.75" thickBot="1">
+    <row r="2" ht="99.75" customHeight="1">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -787,7 +810,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="99.75" thickBot="1">
+    <row r="3" ht="99.75" customHeight="1">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -804,7 +827,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="116.25" thickBot="1">
+    <row r="4" ht="116.25" customHeight="1">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -821,7 +844,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="116.25" thickBot="1">
+    <row r="5" ht="116.25" customHeight="1">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -838,7 +861,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="99.75" thickBot="1">
+    <row r="6" ht="99.75" customHeight="1">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -855,7 +878,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="50.25" thickBot="1">
+    <row r="7" ht="50.25" customHeight="1">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -872,7 +895,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="99.75" thickBot="1">
+    <row r="8" ht="99.75" customHeight="1">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -889,7 +912,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="66.75" thickBot="1">
+    <row r="9" ht="66.75" customHeight="1">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -906,7 +929,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="132.75" thickBot="1">
+    <row r="10" ht="132.75" customHeight="1">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -923,7 +946,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="66.75" thickBot="1">
+    <row r="11" ht="66.75" customHeight="1">
       <c r="A11" s="2">
         <v>10</v>
       </c>
@@ -940,7 +963,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="99.75" thickBot="1">
+    <row r="12" ht="99.75" customHeight="1">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -957,7 +980,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="83.25" thickBot="1">
+    <row r="13" ht="83.25" customHeight="1">
       <c r="A13" s="2">
         <v>12</v>
       </c>
@@ -974,7 +997,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="99.75" thickBot="1">
+    <row r="14" ht="99.75" customHeight="1">
       <c r="A14" s="2">
         <v>13</v>
       </c>
@@ -991,7 +1014,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="149.25" thickBot="1">
+    <row r="15" ht="149.25" customHeight="1">
       <c r="A15" s="2">
         <v>14</v>
       </c>
@@ -1008,7 +1031,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="99.75" thickBot="1">
+    <row r="16" ht="99.75" customHeight="1">
       <c r="A16" s="2">
         <v>15</v>
       </c>
@@ -1025,7 +1048,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="17" spans="1:5" ht="132.75" thickBot="1">
+    <row r="17" ht="132.75" customHeight="1">
       <c r="A17" s="2">
         <v>16</v>
       </c>
@@ -1042,7 +1065,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="18" spans="1:5" ht="132.75" thickBot="1">
+    <row r="18" ht="132.75" customHeight="1">
       <c r="A18" s="2">
         <v>17</v>
       </c>
@@ -1059,7 +1082,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="19" spans="1:5" ht="83.25" thickBot="1">
+    <row r="19" ht="83.25" customHeight="1">
       <c r="A19" s="2">
         <v>18</v>
       </c>
@@ -1076,7 +1099,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="20" spans="1:5" ht="132.75" thickBot="1">
+    <row r="20" ht="132.75" customHeight="1">
       <c r="A20" s="2">
         <v>19</v>
       </c>
@@ -1093,7 +1116,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="21" spans="1:5" ht="83.25" thickBot="1">
+    <row r="21" ht="83.25" customHeight="1">
       <c r="A21" s="2">
         <v>20</v>
       </c>
@@ -1110,7 +1133,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="22" spans="1:5" ht="99.75" thickBot="1">
+    <row r="22" ht="99.75" customHeight="1">
       <c r="A22" s="2">
         <v>21</v>
       </c>
@@ -1127,7 +1150,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="23" spans="1:5" ht="66.75" thickBot="1">
+    <row r="23" ht="66.75" customHeight="1">
       <c r="A23" s="2">
         <v>22</v>
       </c>
@@ -1144,7 +1167,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="24" spans="1:5" ht="99.75" thickBot="1">
+    <row r="24" ht="99.75" customHeight="1">
       <c r="A24" s="2">
         <v>23</v>
       </c>
@@ -1161,7 +1184,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="25" spans="1:5" ht="83.25" thickBot="1">
+    <row r="25" ht="83.25" customHeight="1">
       <c r="A25" s="2">
         <v>24</v>
       </c>
@@ -1178,7 +1201,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="26" spans="1:5" ht="66.75" thickBot="1">
+    <row r="26" ht="66.75" customHeight="1">
       <c r="A26" s="2">
         <v>25</v>
       </c>
@@ -1195,7 +1218,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="27" spans="1:5" ht="66.75" thickBot="1">
+    <row r="27" ht="66.75" customHeight="1">
       <c r="A27" s="2">
         <v>26</v>
       </c>
@@ -1212,7 +1235,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="28" spans="1:5" ht="83.25" thickBot="1">
+    <row r="28" ht="83.25" customHeight="1">
       <c r="A28" s="2">
         <v>27</v>
       </c>
@@ -1229,7 +1252,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="29" spans="1:5" ht="99.75" thickBot="1">
+    <row r="29" ht="99.75" customHeight="1">
       <c r="A29" s="2">
         <v>28</v>
       </c>
@@ -1246,7 +1269,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="30" spans="1:5" ht="83.25" thickBot="1">
+    <row r="30" ht="83.25" customHeight="1">
       <c r="A30" s="2">
         <v>29</v>
       </c>
@@ -1263,7 +1286,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="31" spans="1:5" ht="132.75" thickBot="1">
+    <row r="31" ht="132.75" customHeight="1">
       <c r="A31" s="2">
         <v>30</v>
       </c>
@@ -1280,7 +1303,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="32" spans="1:5" ht="83.25" thickBot="1">
+    <row r="32" ht="83.25" customHeight="1">
       <c r="A32" s="2">
         <v>31</v>
       </c>
@@ -1297,7 +1320,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="33" spans="1:5" ht="99.75" thickBot="1">
+    <row r="33" ht="99.75" customHeight="1">
       <c r="A33" s="2">
         <v>32</v>
       </c>
@@ -1314,7 +1337,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="34" spans="1:5" ht="99.75" thickBot="1">
+    <row r="34" ht="99.75" customHeight="1">
       <c r="A34" s="2">
         <v>33</v>
       </c>
@@ -1331,7 +1354,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="35" spans="1:5" ht="83.25" thickBot="1">
+    <row r="35" ht="83.25" customHeight="1">
       <c r="A35" s="2">
         <v>34</v>
       </c>
@@ -1348,7 +1371,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="36" spans="1:5" ht="99.75" thickBot="1">
+    <row r="36" ht="99.75" customHeight="1">
       <c r="A36" s="2">
         <v>35</v>
       </c>
@@ -1365,7 +1388,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="37" spans="1:5" ht="99.75" thickBot="1">
+    <row r="37" ht="99.75" customHeight="1">
       <c r="A37" s="2">
         <v>36</v>
       </c>
@@ -1382,7 +1405,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="38" spans="1:5" ht="66.75" thickBot="1">
+    <row r="38" ht="66.75" customHeight="1">
       <c r="A38" s="2">
         <v>37</v>
       </c>
@@ -1399,7 +1422,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="39" spans="1:5" ht="50.25" thickBot="1">
+    <row r="39" ht="50.25" customHeight="1">
       <c r="A39" s="2">
         <v>38</v>
       </c>
@@ -1416,7 +1439,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="40" spans="1:5" ht="83.25" thickBot="1">
+    <row r="40" ht="83.25" customHeight="1">
       <c r="A40" s="2">
         <v>39</v>
       </c>
@@ -1433,7 +1456,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="41" spans="1:5" ht="66.75" thickBot="1">
+    <row r="41" ht="66.75" customHeight="1">
       <c r="A41" s="2">
         <v>40</v>
       </c>
@@ -1450,7 +1473,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="42" spans="1:5" ht="83.25" thickBot="1">
+    <row r="42" ht="83.25" customHeight="1">
       <c r="A42" s="2">
         <v>41</v>
       </c>
@@ -1467,7 +1490,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="43" spans="1:5" ht="66.75" thickBot="1">
+    <row r="43" ht="66.75" customHeight="1">
       <c r="A43" s="2">
         <v>42</v>
       </c>
@@ -1484,7 +1507,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="44" spans="1:5" ht="132.75" thickBot="1">
+    <row r="44" ht="132.75" customHeight="1">
       <c r="A44" s="2">
         <v>43</v>
       </c>
@@ -1501,7 +1524,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="45" spans="1:5" ht="66.75" thickBot="1">
+    <row r="45" ht="66.75" customHeight="1">
       <c r="A45" s="2">
         <v>44</v>
       </c>
@@ -1518,7 +1541,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="46" spans="1:5" ht="99.75" thickBot="1">
+    <row r="46" ht="99.75" customHeight="1">
       <c r="A46" s="2">
         <v>45</v>
       </c>
@@ -1535,7 +1558,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="47" spans="1:5" ht="83.25" thickBot="1">
+    <row r="47" ht="83.25" customHeight="1">
       <c r="A47" s="2">
         <v>46</v>
       </c>
@@ -1552,7 +1575,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="48" spans="1:5" ht="66.75" thickBot="1">
+    <row r="48" ht="66.75" customHeight="1">
       <c r="A48" s="2">
         <v>47</v>
       </c>
@@ -1569,7 +1592,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="49" spans="1:5" ht="66.75" thickBot="1">
+    <row r="49" ht="66.75" customHeight="1">
       <c r="A49" s="2">
         <v>48</v>
       </c>
@@ -1586,7 +1609,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="50" spans="1:5" ht="83.25" thickBot="1">
+    <row r="50" ht="83.25" customHeight="1">
       <c r="A50" s="2">
         <v>49</v>
       </c>
@@ -1603,7 +1626,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="51" spans="1:5" ht="99.75" thickBot="1">
+    <row r="51" ht="99.75" customHeight="1">
       <c r="A51" s="2">
         <v>50</v>
       </c>
@@ -1620,7 +1643,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="52" spans="1:5" ht="116.25" thickBot="1">
+    <row r="52" ht="116.25" customHeight="1">
       <c r="A52" s="2">
         <v>51</v>
       </c>
@@ -1637,7 +1660,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="53" spans="1:5" ht="149.25" thickBot="1">
+    <row r="53" ht="149.25" customHeight="1">
       <c r="A53" s="2">
         <v>52</v>
       </c>
@@ -1654,7 +1677,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="54" spans="1:5" ht="66.75" thickBot="1">
+    <row r="54" ht="66.75" customHeight="1">
       <c r="A54" s="2">
         <v>53</v>
       </c>
@@ -1671,7 +1694,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="55" spans="1:5" ht="99.75" thickBot="1">
+    <row r="55" ht="99.75" customHeight="1">
       <c r="A55" s="2">
         <v>54</v>
       </c>
@@ -1688,7 +1711,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="56" spans="1:5" ht="83.25" thickBot="1">
+    <row r="56" ht="83.25" customHeight="1">
       <c r="A56" s="2">
         <v>55</v>
       </c>
@@ -1705,7 +1728,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="57" spans="1:5" ht="132.75" thickBot="1">
+    <row r="57" ht="132.75" customHeight="1">
       <c r="A57" s="2">
         <v>56</v>
       </c>
@@ -1722,7 +1745,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="58" spans="1:5" ht="116.25" thickBot="1">
+    <row r="58" ht="116.25" customHeight="1">
       <c r="A58" s="2">
         <v>57</v>
       </c>
@@ -1739,7 +1762,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="59" spans="1:5" ht="116.25" thickBot="1">
+    <row r="59" ht="116.25" customHeight="1">
       <c r="A59" s="2">
         <v>58</v>
       </c>
@@ -1756,7 +1779,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="60" spans="1:5" ht="99.75" thickBot="1">
+    <row r="60" ht="99.75" customHeight="1">
       <c r="A60" s="2">
         <v>59</v>
       </c>
@@ -1773,7 +1796,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="61" spans="1:5" ht="83.25" thickBot="1">
+    <row r="61" ht="83.25" customHeight="1">
       <c r="A61" s="2">
         <v>60</v>
       </c>
@@ -1790,7 +1813,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="62" spans="1:5" ht="99.75" thickBot="1">
+    <row r="62" ht="99.75" customHeight="1">
       <c r="A62" s="2">
         <v>61</v>
       </c>
@@ -1807,7 +1830,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="63" spans="1:5" ht="99.75" thickBot="1">
+    <row r="63" ht="99.75" customHeight="1">
       <c r="A63" s="2">
         <v>62</v>
       </c>
@@ -1824,7 +1847,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="64" spans="1:5" ht="99.75" thickBot="1">
+    <row r="64" ht="99.75" customHeight="1">
       <c r="A64" s="2">
         <v>63</v>
       </c>
@@ -1841,7 +1864,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="65" spans="1:5" ht="116.25" thickBot="1">
+    <row r="65" ht="116.25" customHeight="1">
       <c r="A65" s="2">
         <v>64</v>
       </c>
@@ -1858,7 +1881,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="66" spans="1:5" ht="116.25" thickBot="1">
+    <row r="66" ht="116.25" customHeight="1">
       <c r="A66" s="2">
         <v>65</v>
       </c>
@@ -1875,7 +1898,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="67" spans="1:5" ht="66.75" thickBot="1">
+    <row r="67" ht="66.75" customHeight="1">
       <c r="A67" s="2">
         <v>66</v>
       </c>
@@ -1892,7 +1915,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="68" spans="1:5" ht="132.75" thickBot="1">
+    <row r="68" ht="132.75" customHeight="1">
       <c r="A68" s="2">
         <v>67</v>
       </c>
@@ -1909,7 +1932,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="69" spans="1:5" ht="66.75" thickBot="1">
+    <row r="69" ht="66.75" customHeight="1">
       <c r="A69" s="2">
         <v>68</v>
       </c>
@@ -1926,7 +1949,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="70" spans="1:5" ht="116.25" thickBot="1">
+    <row r="70" ht="116.25" customHeight="1">
       <c r="A70" s="2">
         <v>69</v>
       </c>
@@ -1943,7 +1966,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="71" spans="1:5" ht="99.75" thickBot="1">
+    <row r="71" ht="99.75" customHeight="1">
       <c r="A71" s="2">
         <v>70</v>
       </c>
@@ -1960,7 +1983,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="72" spans="1:5" ht="116.25" thickBot="1">
+    <row r="72" ht="116.25" customHeight="1">
       <c r="A72" s="2">
         <v>71</v>
       </c>
@@ -1977,7 +2000,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="73" spans="1:5" ht="116.25" thickBot="1">
+    <row r="73" ht="116.25" customHeight="1">
       <c r="A73" s="2">
         <v>72</v>
       </c>
@@ -1994,7 +2017,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="74" spans="1:5" ht="99.75" thickBot="1">
+    <row r="74" ht="99.75" customHeight="1">
       <c r="A74" s="2">
         <v>73</v>
       </c>
@@ -2011,7 +2034,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="75" spans="1:5" ht="116.25" thickBot="1">
+    <row r="75" ht="116.25" customHeight="1">
       <c r="A75" s="2">
         <v>74</v>
       </c>
@@ -2028,7 +2051,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="76" spans="1:5" ht="132.75" thickBot="1">
+    <row r="76" ht="132.75" customHeight="1">
       <c r="A76" s="2">
         <v>75</v>
       </c>
@@ -2046,8 +2069,13 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="3" type="noConversion"/>
+  <printOptions/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" pageOrder="downThenOver" orientation="portrait"/>
+  <headerFooter>
+    <oddHeader>&amp;L&amp;C&amp;R</oddHeader>
+    <oddFooter>&amp;L&amp;C&amp;R</oddFooter>
+  </headerFooter>
+  <extLst/>
 </worksheet>
 </file>
</xml_diff>